<commit_message>
Latest changes: menu import fixes, remove Edit Menu from nav, etc.
</commit_message>
<xml_diff>
--- a/data/Latest_Update/Client Vlaidated Pricing/NC Pricing ΓÇö Non-Veg Menu1.xlsx
+++ b/data/Latest_Update/Client Vlaidated Pricing/NC Pricing ΓÇö Non-Veg Menu1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24109080beb0ba33/Hi-Tech Foods LLC/Catering Software/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nidhi-catering-oms-FULL-DEPLOYMENT\data\Latest_Update\Client Vlaidated Pricing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{39CD1536-9FA5-4139-9601-A1907A61C3DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83B8B909-C4D5-4DDA-B7AA-AF23421B5F10}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52297D0F-FBF5-4B7D-959A-E8A487AC94EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Non-Veg Menu'!$A$2:$I$134</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -878,7 +878,7 @@
     <col min="9" max="9" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="28" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>

</xml_diff>